<commit_message>
Update dataset and recommend logic
</commit_message>
<xml_diff>
--- a/Dataset/Jenis Kulit Cocok.xlsx
+++ b/Dataset/Jenis Kulit Cocok.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TAGw\backend\Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E055F5BF-7911-4C55-B9B4-68A2ABFD2BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B2D1CC-5A84-4AC4-8979-150F0FF2B596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3516" uniqueCount="1777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3522" uniqueCount="1779">
   <si>
     <t>Jenis_Kulit</t>
   </si>
@@ -5351,6 +5351,12 @@
   </si>
   <si>
     <t>Sangat ideal untuk mereduksi produksi minyak berlebih di area T-zone secara terfokus tanpa membebani area pipi secara fluktuatif.</t>
+  </si>
+  <si>
+    <t>Memiliki konsistensi yang cukup padat dan berat (heavy feel). Pada kulit yang memproduksi banyak minyak, bahan ini akan terasa sangat pengap, lengket, dan memperparah kilap sebum di wajah.</t>
+  </si>
+  <si>
+    <t>Berpotensi meninggalkan lapisan oklusif tebal yang dapat menyumbat folikel pilosebasea aktif di area T-zone.</t>
   </si>
 </sst>
 </file>
@@ -42065,9 +42071,15 @@
       <c r="W1174" s="2"/>
     </row>
     <row r="1175" spans="1:23" ht="15.75" customHeight="1">
-      <c r="A1175" s="7"/>
-      <c r="B1175" s="7"/>
-      <c r="C1175" s="7"/>
+      <c r="A1175" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1175" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="C1175" s="6" t="s">
+        <v>1777</v>
+      </c>
       <c r="D1175" s="2"/>
       <c r="E1175" s="2"/>
       <c r="F1175" s="2"/>
@@ -42090,9 +42102,15 @@
       <c r="W1175" s="2"/>
     </row>
     <row r="1176" spans="1:23" ht="15.75" customHeight="1">
-      <c r="A1176" s="7"/>
-      <c r="B1176" s="7"/>
-      <c r="C1176" s="7"/>
+      <c r="A1176" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1176" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="C1176" s="6" t="s">
+        <v>1778</v>
+      </c>
       <c r="D1176" s="2"/>
       <c r="E1176" s="2"/>
       <c r="F1176" s="2"/>

</xml_diff>